<commit_message>
chore: run 2026-04-21 11:11 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_21_04_2026.xlsx
+++ b/logs/Consolidado_21_04_2026.xlsx
@@ -620,10 +620,10 @@
         <v>152</v>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -639,10 +639,10 @@
         <v>65</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -677,10 +677,10 @@
         <v>69</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -715,10 +715,10 @@
         <v>100</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>4</v>
@@ -970,40 +970,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Antirougeurs DAY Soothing Emulsion
 Emulsão Antivermelhidão Pele Mista SPF30
 40 ml</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/antirougeurs-day-soothing-emulsion-4878505.html</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>4878505</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -2984,40 +2984,40 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Dermabsolu Eco-Refill Redensifying Day Cream
 Recarga Creme anti idade Rugas e Firmeza
 50 ml</t>
         </is>
       </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/dermabsolu-eco-refill-redensifying-day-cream-8152747.html</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr"/>
-      <c r="F56" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>8152747</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -3132,7 +3132,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr"/>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>6739604</t>
+        </is>
+      </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
           <t>30%</t>
@@ -3340,40 +3344,40 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C65" s="7" t="inlineStr">
         <is>
           <t>Hyaluron Activ B3 Coffret de Natal
 Coffret Sérum Rugas Ácido Hialurónico Niacinamida
 1 un</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/hyaluron-activ-b3-coffret-de-natal-8608333.html</t>
         </is>
       </c>
-      <c r="E65" s="5" t="inlineStr"/>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr">
+      <c r="E65" s="7" t="inlineStr"/>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
         <is>
           <t>8608333</t>
         </is>
       </c>
-      <c r="H65" s="5" t="inlineStr">
+      <c r="H65" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -8698,40 +8702,40 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Kelual Squanorm Anti-Dandruff Refresh Lotion
 Loção Leave-in Refrescante Cabelo com Caspa
 190 ml</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/kelual-squanorm-anti-dandruff-refresh-lotion-8660190.html</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr"/>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>8660190</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -12081,40 +12085,40 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Style Modeling Paste
 Pasta para Cabelo Modeladora Fixação Natural
 75 ml</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/style-modeling-paste-7447301.html</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>7447301</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -12281,40 +12285,40 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>Sublime Curl Activating Spray Wavy Curly Hair
 Spray Cabelo Leave-In Redefinidor de Caracóis
 150 ml</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sublime-curl-activating-spray-wavy-curly-hair-6490914.html</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
         <is>
           <t>6490914</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H50" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -18431,40 +18435,40 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>Elgydium
 Fio Dentário Crossing Floss
 1 un</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/fio-dentario-crossing-floss-8099110.html</t>
         </is>
       </c>
-      <c r="E62" s="3" t="inlineStr"/>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
+      <c r="E62" s="7" t="inlineStr"/>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>8099110</t>
         </is>
       </c>
-      <c r="H62" s="3" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -18993,17 +18997,17 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B76" s="7" t="inlineStr">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C76" s="7" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>Eludril
 Ortho Colutório Uso Diário
@@ -19011,23 +19015,23 @@
 500 ml</t>
         </is>
       </c>
-      <c r="D76" s="7" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/ortho-colutorio-uso-diario-7631910.html</t>
         </is>
       </c>
-      <c r="E76" s="7" t="inlineStr"/>
-      <c r="F76" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G76" s="7" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr"/>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
         <is>
           <t>7631910</t>
         </is>
       </c>
-      <c r="H76" s="7" t="inlineStr">
+      <c r="H76" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -19314,40 +19318,40 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="7" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B84" s="7" t="inlineStr">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C84" s="7" t="inlineStr">
+      <c r="C84" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Pasta Dentrífica Júnior Tutti Fruti Emoji
 50 ml</t>
         </is>
       </c>
-      <c r="D84" s="7" t="inlineStr">
+      <c r="D84" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/pasta-dentrifica-junior-tutti-fruti-emoji-7607823.html</t>
         </is>
       </c>
-      <c r="E84" s="7" t="inlineStr"/>
-      <c r="F84" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G84" s="7" t="inlineStr">
+      <c r="E84" s="3" t="inlineStr"/>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
         <is>
           <t>7607823</t>
         </is>
       </c>
-      <c r="H84" s="7" t="inlineStr">
+      <c r="H84" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>

</xml_diff>

<commit_message>
chore: run 2026-04-21 15:15 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_21_04_2026.xlsx
+++ b/logs/Consolidado_21_04_2026.xlsx
@@ -10,11 +10,12 @@
     <sheet name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Avène" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Ducray" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="René Furterer" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="A-Derma" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Oral Care" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Dexeryl" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Variantes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Klorane" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="René Furterer" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="A-Derma" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Oral Care" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dexeryl" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Variantes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -217,7 +218,24 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Marca_René_Furterer" displayName="Marca_René_Furterer" ref="A1:H74" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Marca_Klorane" displayName="Marca_Klorane" ref="A1:H35" headerRowCount="1">
+  <autoFilter ref="A1:H35"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="data"/>
+    <tableColumn id="2" name="marca"/>
+    <tableColumn id="3" name="titulo"/>
+    <tableColumn id="4" name="url"/>
+    <tableColumn id="5" name="nome_variante"/>
+    <tableColumn id="6" name="is_oos"/>
+    <tableColumn id="7" name="ref_produto"/>
+    <tableColumn id="8" name="desconto"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Marca_René_Furterer" displayName="Marca_René_Furterer" ref="A1:H74" headerRowCount="1">
   <autoFilter ref="A1:H74"/>
   <tableColumns count="8">
     <tableColumn id="1" name="data"/>
@@ -233,8 +251,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Marca_A_Derma" displayName="Marca_A_Derma" ref="A1:H64" headerRowCount="1">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Marca_A_Derma" displayName="Marca_A_Derma" ref="A1:H64" headerRowCount="1">
   <autoFilter ref="A1:H64"/>
   <tableColumns count="8">
     <tableColumn id="1" name="data"/>
@@ -250,8 +268,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Marca_Oral_Care" displayName="Marca_Oral_Care" ref="A1:H101" headerRowCount="1">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Marca_Oral_Care" displayName="Marca_Oral_Care" ref="A1:H101" headerRowCount="1">
   <autoFilter ref="A1:H101"/>
   <tableColumns count="8">
     <tableColumn id="1" name="data"/>
@@ -267,8 +285,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Marca_Dexeryl" displayName="Marca_Dexeryl" ref="A1:H10" headerRowCount="1">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Marca_Dexeryl" displayName="Marca_Dexeryl" ref="A1:H10" headerRowCount="1">
   <autoFilter ref="A1:H10"/>
   <tableColumns count="8">
     <tableColumn id="1" name="data"/>
@@ -623,7 +641,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -655,10 +673,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -718,7 +736,7 @@
         <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>4</v>
@@ -10295,6 +10313,1476 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>marca</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>nome_variante</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>is_oos</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>ref_produto</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>desconto</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Bebé Cleansing Lotion No-Rise
+Leite Limpeza Fralda e Mãos 0 meses
+500 ml</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/bebe-cleansing-lotion-no-rise-6661598.html</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>6661598</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Bebé Multi-Purpose Oil BIO
+Óleo Multiusos BIO Limpa Nutre desde 0 meses
+200 ml</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/bebe-multi-purpose-oil-bio-7831747.html</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>7831747</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Centaury Anti-Yellowing Gray, Blond Shampoo
+Champô Centáurea BIO Neutraliza Tons Amarelos
+400 ml</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/centaury-anti-yellowing-gray-blond-shampoo-6863851.html</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>6863851</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Chamomile Brightening Blond Hair Spray
+Spray Camomila Aclarador 3-em-1 Cabelo Loiro
+100 ml</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/chamomile-brightening-blond-hair-spray-7615327.html</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>7615327</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Eau de Parfumee e Oferta de Coelho
+1 un</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/eau-de-parfumee-e-oferta-de-coelho-6661579.html</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>6661579</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Flax Volume Fine Hair Conditioner
+Condicionador Linho BIO Volume Cabelo Fino
+200 ml</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/flax-volume-fine-hair-conditioner-5924193.html</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>5924193</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Galanga Anti-Dandruff Anti-itching Treatment
+Loção Anti Caspa Tratamento Anti-comichão
+100 ml</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/galanga-anti-dandruff-anti-itching-treatment-8544717.html</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>8544717</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Galanga Anti-Dandruff Shampoo
+Champô Anti Caspa Reequilibra e Trata</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/galanga-anti-dandruff-shampoo-427225.html</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>8544713</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Galanga Anti-Dandruff Shampoo
+Champô Anti Caspa Reequilibra e Trata</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/galanga-anti-dandruff-shampoo-427225.html</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>400 ml</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>8544715</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Gel Lavante Suave Bebé
+500 ml</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/gel-lavante-suave-bebe-6661468.html</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>6661468</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Carolina Herrera
+Good Girl Jasmine Absolute Eau de Parfum
+Perfume para Mulher</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/good-girl-jasmine-absolute-eau-de-parfum-453824.html</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>30 ml</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>8795826</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Carolina Herrera
+Good Girl Jasmine Absolute Eau de Parfum
+Perfume para Mulher</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/good-girl-jasmine-absolute-eau-de-parfum-453824.html</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>80 ml</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>8795828</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Carolina Herrera
+Good Girl Jasmine Absolute Eau de Parfum
+Perfume para Mulher</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/good-girl-jasmine-absolute-eau-de-parfum-453824.html</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>8795830</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Hair Removal Cream Sweet Almond
+Creme Depilatório pele Sensível Amêndoas Doce
+150 ml</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/hair-removal-cream-sweet-almond-7724355.html</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>7724355</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Huile Sèche Solaire SPF 30
+Protetor Solar de Corpo e Cabelo
+200 ml</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/huile-seche-solaire-spf-30-7129222.html</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>7129222</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Junior Detangling Shampoo
+Champô de Pêssego a partir de 3 anos
+500 ml</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/junior-detangling-shampoo-3066288.html</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>3066288</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Vichy
+Liftactiv Collagen Specialist 16 Serum
+Sérum Rosto para Sinais de Envelhecimento
+30 ml</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/liftactiv-collagen-specialist-16-serum-8377324.html</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>8377324</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Mango Nourishing Leave-In Cream
+Creme Dia Manga Nutritivo SOS Cabelo Seco
+125ml</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/mango-nourishing-leave-in-cream-5072223.html</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>5072223</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Mango Nourishing Mask
+Máscara Manga Nutritiva Hidrata Cabelo Seco
+250 ml</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/mango-nourishing-mask-3066267.html</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>3066267</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Mango Nourishing Shampoo
+Champô Manga Nutritivo para Cabelo Seco</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>3018059</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Mango Nourishing Shampoo
+Champô Manga Nutritivo para Cabelo Seco</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>400 ml</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>3066184</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Mango Nourishing Shampoo
+Champô Manga Nutritivo para Cabelo Seco</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>100 ml</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>6128309</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Nettle &amp; Clay 2-in-1 Mask Shampoo
+Máscara Champô Pó Ortiga BIO Cabelo Oleoso
+150 ml</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/nettle-and-clay-2-in-1-mask-shampoo-7339155.html</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>7339155</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Oat Ultra-Gentle All HairTypes Conditioner
+Condicionador Aveia Suave e Protetor
+200 ml</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/oat-ultra-gentle-all-hairtypes-conditioner-5924188.html</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>5924188</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Oat&amp;Ceramide Ultra-Gentle Dry Shampoo Dark
+Champô Seco Aveia Ultra-Suave Cabelo Castanho</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>https://wells.pt/oatandceramide-ultra-gentle-dry-shampoo-dark-341982.html</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>7831154</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Oat&amp;Ceramide Ultra-Gentle Dry Shampoo Dark
+Champô Seco Aveia Ultra-Suave Cabelo Castanho</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/oatandceramide-ultra-gentle-dry-shampoo-dark-341982.html</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>150 ml</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>7831155</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Pivoine Apaisant &amp; Anti-Irritant Aprés-Shampooing
+Gel Calmante Pós-champô Perfumado
+150 ml</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/pivoine-apaisant-and-anti-irritant-apres-shampooing-6308308.html</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>6308308</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Prickly Pear 24h Hydration &amp; Shine Sérum
+Sérum Figo da índia Hidrata Ácido Hialurónico
+100 ml</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/prickly-pear-24h-hydration-and-shine-serum-8067444.html</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>8067444</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Prickly Pear 72h Hydration&amp;Shine Plump Mask
+Máscara Figo da índia Hidrata 72h Cabelo Baço
+250 ml</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/prickly-pear-72h-hydrationandshine-plump-mask-8067433.html</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>8067433</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Quinine Anti-Hair Loss Intense Strengthening
+Sérum Quinina Queda de Cabelo e Força
+100 ml</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/quinine-anti-hair-loss-intense-strengthening-8423056.html</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>8423056</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Quinine Strengthening Thinning Hair Shampoo
+Champô Fortificante e Revitalizante Antiqueda</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/quinine-strengthening-thinning-hair-shampoo-343977.html</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>400 ml</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>3000714</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Quinine Strengthening Thinning Hair Shampoo
+Champô Fortificante e Revitalizante Antiqueda</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/quinine-strengthening-thinning-hair-shampoo-343977.html</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>3000716</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Quinine Strengthening Thinning Hair Shampoo
+Champô Fortificante e Revitalizante Antiqueda</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/quinine-strengthening-thinning-hair-shampoo-343977.html</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>100 ml</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>4468119</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Tamanu BIO e Monoi Spray Solar Sublime SPF30
+Protetor Solar Spray Corpo Sublimador
+200 ml</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/tamanu-bio-e-monoi-spray-solar-sublime-spf30-7129223.html</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr"/>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>7129223</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -13298,7 +14786,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13548,11 +15036,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>7756107</t>
-        </is>
-      </c>
+      <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>25%</t>
@@ -15962,7 +17446,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20059,7 +21543,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20498,13 +21982,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -22835,264 +24319,761 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Carolina Herrera
+Good Girl Jasmine Absolute Eau de Parfum
+Perfume para Mulher</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>30 ml</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>8795826</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/good-girl-jasmine-absolute-eau-de-parfum-453824.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Carolina Herrera
+Good Girl Jasmine Absolute Eau de Parfum
+Perfume para Mulher</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>8795830</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/good-girl-jasmine-absolute-eau-de-parfum-453824.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Carolina Herrera
+Good Girl Jasmine Absolute Eau de Parfum
+Perfume para Mulher</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>80 ml</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>8795828</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/good-girl-jasmine-absolute-eau-de-parfum-453824.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Galanga Anti-Dandruff Shampoo
+Champô Anti Caspa Reequilibra e Trata</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>8544713</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/galanga-anti-dandruff-shampoo-427225.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Galanga Anti-Dandruff Shampoo
+Champô Anti Caspa Reequilibra e Trata</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>400 ml</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>8544715</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/galanga-anti-dandruff-shampoo-427225.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Mango Nourishing Shampoo
+Champô Manga Nutritivo para Cabelo Seco</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>100 ml</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>6128309</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Mango Nourishing Shampoo
+Champô Manga Nutritivo para Cabelo Seco</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>3018059</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Mango Nourishing Shampoo
+Champô Manga Nutritivo para Cabelo Seco</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>400 ml</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>3066184</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Oat&amp;Ceramide Ultra-Gentle Dry Shampoo Dark
+Champô Seco Aveia Ultra-Suave Cabelo Castanho</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>150 ml</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>7831155</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>https://wells.pt/oatandceramide-ultra-gentle-dry-shampoo-dark-341982.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Oat&amp;Ceramide Ultra-Gentle Dry Shampoo Dark
+Champô Seco Aveia Ultra-Suave Cabelo Castanho</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>7831154</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>https://wells.pt/oatandceramide-ultra-gentle-dry-shampoo-dark-341982.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Quinine Strengthening Thinning Hair Shampoo
+Champô Fortificante e Revitalizante Antiqueda</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>100 ml</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>4468119</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/quinine-strengthening-thinning-hair-shampoo-343977.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Quinine Strengthening Thinning Hair Shampoo
+Champô Fortificante e Revitalizante Antiqueda</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>3000716</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/quinine-strengthening-thinning-hair-shampoo-343977.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Klorane</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Quinine Strengthening Thinning Hair Shampoo
+Champô Fortificante e Revitalizante Antiqueda</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>400 ml</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>3000714</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>https://wells.pt/quinine-strengthening-thinning-hair-shampoo-343977.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>Forticea Strengthening Revitalizing Shampoo
 Champô Fortificante Todos Tipos de Cabelo</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>250ml</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
         <is>
           <t>6759973</t>
         </is>
       </c>
-      <c r="F62" s="3" t="inlineStr">
+      <c r="F75" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="G62" s="3" t="inlineStr">
+      <c r="G75" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/forticea-strengthening-revitalizing-shampoo-343991.html</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B76" s="5" t="inlineStr">
         <is>
           <t>Forticea Strengthening Revitalizing Shampoo
 Champô Fortificante Todos Tipos de Cabelo</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
         <is>
           <t>7630905</t>
         </is>
       </c>
-      <c r="F63" s="3" t="inlineStr">
+      <c r="F76" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="G76" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/forticea-strengthening-revitalizing-shampoo-343991.html</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B64" s="5" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>Naturia Gentle Micellair Shampoo
 Champô Suave Uso Frequente e Familiar</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
         <is>
           <t>6633968</t>
         </is>
       </c>
-      <c r="F64" s="5" t="inlineStr">
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G64" s="5" t="inlineStr">
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/naturia-gentle-micellair-shampoo-343992.html</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
         <is>
           <t>Naturia Gentle Micellair Shampoo
 Champô Suave Uso Frequente e Familiar</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
         <is>
           <t>7610972</t>
         </is>
       </c>
-      <c r="F65" s="5" t="inlineStr">
+      <c r="F78" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="G65" s="5" t="inlineStr">
+      <c r="G78" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/naturia-gentle-micellair-shampoo-343992.html</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B66" s="5" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>Naturia Gentle Micellair Shampoo
 Champô Suave Uso Frequente e Familiar</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
         <is>
           <t>5522799</t>
         </is>
       </c>
-      <c r="F66" s="5" t="inlineStr">
+      <c r="F79" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G66" s="5" t="inlineStr">
+      <c r="G79" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/naturia-gentle-micellair-shampoo-343992.html</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B80" s="5" t="inlineStr">
         <is>
           <t>Triphasic Active Grow Shampoo
 Champô Crescimento do Cabelo</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
         <is>
           <t>8557861</t>
         </is>
       </c>
-      <c r="F67" s="3" t="inlineStr">
+      <c r="F80" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G67" s="3" t="inlineStr">
+      <c r="G80" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-active-grow-shampoo-427541.html</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B81" s="5" t="inlineStr">
         <is>
           <t>Triphasic Active Grow Shampoo
 Champô Crescimento do Cabelo</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C81" s="5" t="inlineStr">
         <is>
           <t>500 ml</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
         <is>
           <t>8557868</t>
         </is>
       </c>
-      <c r="F68" s="3" t="inlineStr">
+      <c r="F81" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G68" s="3" t="inlineStr">
+      <c r="G81" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-active-grow-shampoo-427541.html</t>
         </is>

</xml_diff>